<commit_message>
fix tamplate lampiran lembur
</commit_message>
<xml_diff>
--- a/src/templates/Lampiran_Lembur.xlsx
+++ b/src/templates/Lampiran_Lembur.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomat/Developer/apiAbsen/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{639B72DB-D077-6040-B117-E30B4037A64C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B413002-C57A-914D-868E-274C245B293D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="21860" windowHeight="14940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,10 +56,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0.00000000000"/>
-    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -102,26 +98,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -458,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -505,54 +486,6 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-    </row>
   </sheetData>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>